<commit_message>
Refractor code for readability/consistency across models and completed dashboard
</commit_message>
<xml_diff>
--- a/Result Tables/Ablation_Temporal_Results.xlsx
+++ b/Result Tables/Ablation_Temporal_Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diogo/dxf243/Result Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609FC8F5-24AC-CD47-8060-238BE0C8437E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C124AD3-1267-844E-A0E6-19245494F1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2700" yWindow="1460" windowWidth="43920" windowHeight="17700" xr2:uid="{59562A5F-441A-104A-93A9-000E75FA76CB}"/>
+    <workbookView xWindow="7880" yWindow="960" windowWidth="31220" windowHeight="15720" xr2:uid="{59562A5F-441A-104A-93A9-000E75FA76CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="80">
   <si>
     <t>FEATURE_NAME</t>
   </si>
@@ -200,9 +200,6 @@
     <t>TestYears</t>
   </si>
   <si>
-    <t>2015 2016</t>
-  </si>
-  <si>
     <t>Accuracy</t>
   </si>
   <si>
@@ -212,9 +209,6 @@
     <t>Features</t>
   </si>
   <si>
-    <t>PR-AUC</t>
-  </si>
-  <si>
     <t>MICRO_ONLY</t>
   </si>
   <si>
@@ -233,40 +227,10 @@
     <t>[2012,2013,2014,2015]</t>
   </si>
   <si>
-    <t>2013,2014, 2015</t>
-  </si>
-  <si>
-    <t>2013, 2014</t>
-  </si>
-  <si>
-    <t>2013, 2014, 2015, 2016</t>
-  </si>
-  <si>
-    <t>2014, 2015</t>
-  </si>
-  <si>
-    <t>2014, 2015, 2016</t>
-  </si>
-  <si>
-    <t>2015, 2016</t>
-  </si>
-  <si>
     <t>Returns Volatility Classification</t>
   </si>
   <si>
     <t>PR_AUC</t>
-  </si>
-  <si>
-    <t>2013, 2014, 2015</t>
-  </si>
-  <si>
-    <t>2014</t>
-  </si>
-  <si>
-    <t>2014 2015</t>
-  </si>
-  <si>
-    <t>2014 2015 2016</t>
   </si>
   <si>
     <t>Volatility Regime Classification</t>
@@ -470,7 +434,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="2" applyBorder="1"/>
@@ -488,9 +452,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -505,7 +466,6 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -525,135 +485,135 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A54AE9C-BD96-4F41-A848-DAB87B5A2992}" name="Table2" displayName="Table2" ref="F3:J12" totalsRowShown="0">
-  <autoFilter ref="F3:J12" xr:uid="{2A54AE9C-BD96-4F41-A848-DAB87B5A2992}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F31EBF09-FEDD-CD4F-A5C5-A22A51D4E341}" name="Features"/>
-    <tableColumn id="2" xr3:uid="{8DC62107-4D2F-314F-AD68-39BB387623F4}" name="Accuracy"/>
-    <tableColumn id="3" xr3:uid="{95E1F2CC-0A25-334E-8EBF-FAA7DE84E622}" name="F1"/>
-    <tableColumn id="4" xr3:uid="{C4B23667-3A2A-EC4C-80D1-66AE7B4847A3}" name="AUC"/>
-    <tableColumn id="5" xr3:uid="{06BFB302-5AA7-5D42-8EF7-61B83701C2FA}" name="PR-AUC"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{FFCDC2A3-A49E-5B49-8C6E-57EADEA7214A}" name="Table7" displayName="Table7" ref="M26:O34" totalsRowShown="0">
+  <autoFilter ref="M26:O34" xr:uid="{FFCDC2A3-A49E-5B49-8C6E-57EADEA7214A}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{EC608A00-87C2-5344-A1ED-7E33F22BD6E8}" name="Features"/>
+    <tableColumn id="2" xr3:uid="{72615F89-B943-7F4F-9727-B2AB56F1FD1D}" name="MAE"/>
+    <tableColumn id="3" xr3:uid="{D3F3DB42-C2D6-B441-8750-C60C10EA5464}" name="RMSE"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{2D3AEF4C-EE0D-8E48-BF01-9511883BF15C}" name="Table11" displayName="Table11" ref="M59:P69" totalsRowShown="0">
-  <autoFilter ref="M59:P69" xr:uid="{2D3AEF4C-EE0D-8E48-BF01-9511883BF15C}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{4799CD6C-3EC4-B947-8D9F-130B15E9530B}" name="TrainYears"/>
-    <tableColumn id="2" xr3:uid="{99938A57-F1EE-9F4D-B06C-244276389F2B}" name="TestYears"/>
-    <tableColumn id="3" xr3:uid="{AB2A9FD9-CA4E-7B4A-847F-0DFA3DFEA2CC}" name="MAE"/>
-    <tableColumn id="4" xr3:uid="{F71AE75F-6746-334F-ABD9-786F60E7B68C}" name="RMSE"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EE3BAF40-C268-4742-AE54-CCAB034D60DE}" name="Table5" displayName="Table5" ref="M13:Q23" totalsRowShown="0">
+  <autoFilter ref="M13:Q23" xr:uid="{EE3BAF40-C268-4742-AE54-CCAB034D60DE}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{C05701D2-283F-8B44-963C-4DA00655C5D8}" name="TrainYears"/>
+    <tableColumn id="2" xr3:uid="{5AD090E9-C625-0344-AE55-11BB16F87225}" name="TestYears"/>
+    <tableColumn id="3" xr3:uid="{0711B295-701C-3B49-87E7-6C9B9AEFBDF4}" name="Accuracy"/>
+    <tableColumn id="4" xr3:uid="{4DAA3220-11DE-B241-AA6F-CAB78CC536A7}" name="Macro_F1"/>
+    <tableColumn id="5" xr3:uid="{29E2D95A-F622-4C47-A9EF-6EF8BC31D48E}" name="Weighted_F1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{48994126-2642-264B-8205-178895D7D1F0}" name="Table3" displayName="Table3" ref="F14:K24" totalsRowShown="0">
-  <autoFilter ref="F14:K24" xr:uid="{48994126-2642-264B-8205-178895D7D1F0}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{A6FC8293-6096-114B-A87A-D16726F83B9D}" name="TrainYears"/>
-    <tableColumn id="2" xr3:uid="{F0938A08-B6A2-9849-AE25-8A70EB38ED90}" name="TestYears" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{73E772F4-B286-1D46-9EC7-D579FE8A4A37}" name="Accuracy"/>
-    <tableColumn id="4" xr3:uid="{C88505F3-A134-CD4E-A4AB-F55520E59240}" name="F1"/>
-    <tableColumn id="5" xr3:uid="{42BEFBE1-DECF-124D-BCB2-C2E6C67DA6E9}" name="AUC"/>
-    <tableColumn id="6" xr3:uid="{F024ED9A-FA0D-154B-9F76-B5E359E1DA5F}" name="PR-AUC" dataDxfId="3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{C9526B9B-25E1-ED45-8A82-DCDB0A7D4782}" name="Table8" displayName="Table8" ref="M36:P46" totalsRowShown="0">
+  <autoFilter ref="M36:P46" xr:uid="{C9526B9B-25E1-ED45-8A82-DCDB0A7D4782}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{30EF76DC-B671-6241-9BDA-587B9EC784D4}" name="TrainYears"/>
+    <tableColumn id="2" xr3:uid="{6A3C4147-2F14-3346-A63B-36802759FC48}" name="TestYears"/>
+    <tableColumn id="3" xr3:uid="{694FA707-6C6B-EB4A-9AE1-A326CF56D236}" name="MAE"/>
+    <tableColumn id="4" xr3:uid="{FFD77189-6482-F944-A4DA-8487DCF8661E}" name="RMSE"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{62B5090D-D872-B24F-B091-1A8E49181E78}" name="Table4" displayName="Table4" ref="F27:J36" totalsRowShown="0">
-  <autoFilter ref="F27:J36" xr:uid="{62B5090D-D872-B24F-B091-1A8E49181E78}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7AC1ED6B-6A35-0E48-B19D-829474A65620}" name="Features"/>
-    <tableColumn id="2" xr3:uid="{FF966BF2-DAFD-B64C-8D0C-E7C08541D1A2}" name="Accuracy"/>
-    <tableColumn id="3" xr3:uid="{3544D75E-21FE-664C-A7D5-0A0B15FCC2FD}" name="F1"/>
-    <tableColumn id="4" xr3:uid="{371143FF-0FCA-CC49-8167-67F9DB68ABFF}" name="AUC"/>
-    <tableColumn id="5" xr3:uid="{8537E7A4-9302-284E-AF64-CC8A039A1FDC}" name="PR_AUC"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B775B231-6629-3E41-9B8A-BD99B10564A8}" name="Table9" displayName="Table9" ref="M49:O57" totalsRowShown="0">
+  <autoFilter ref="M49:O57" xr:uid="{B775B231-6629-3E41-9B8A-BD99B10564A8}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{7923842B-A933-934F-805D-24AC026C4CF8}" name="Features"/>
+    <tableColumn id="2" xr3:uid="{F29B89D6-C129-5A46-84FD-8E90B7466E7C}" name="MAE"/>
+    <tableColumn id="3" xr3:uid="{DF4F34D2-7764-EF4E-B957-842E3FE2F276}" name="RMSE"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EA30ED68-BA33-A94F-86C2-C8D10BD97BA3}" name="Table5" displayName="Table5" ref="F38:K48" totalsRowShown="0">
-  <autoFilter ref="F38:K48" xr:uid="{EA30ED68-BA33-A94F-86C2-C8D10BD97BA3}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{22275962-4554-0D4B-9B76-EA52F29F7482}" name="TrainYears"/>
-    <tableColumn id="2" xr3:uid="{E759CBA5-09BB-794F-8E0F-ACE888AB8D18}" name="TestYears" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{1DF8B83F-497F-1A4A-B2D1-9B1980AAE742}" name="Accuracy"/>
-    <tableColumn id="4" xr3:uid="{0728F650-076E-6148-ADE3-B0E1EA6B2609}" name="F1"/>
-    <tableColumn id="5" xr3:uid="{701D7704-D8DF-384D-8065-1D7E786A707B}" name="AUC"/>
-    <tableColumn id="6" xr3:uid="{D0FE8687-71A1-784F-9D56-B132D4DB5DF9}" name="PR_AUC"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{25A46ADB-9C5F-3F49-BAB9-D73E8D247D92}" name="Table10" displayName="Table10" ref="M59:P69" totalsRowShown="0">
+  <autoFilter ref="M59:P69" xr:uid="{25A46ADB-9C5F-3F49-BAB9-D73E8D247D92}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{B51784BD-84F9-6A4F-B3F3-FEF6D5D99E32}" name="TrainYears"/>
+    <tableColumn id="2" xr3:uid="{E6AF35DD-8A26-6D45-A5FF-57268B6CAFD6}" name="TestYears"/>
+    <tableColumn id="3" xr3:uid="{9E1129EB-ADC8-D349-AB8C-4615997A6F46}" name="MAE"/>
+    <tableColumn id="4" xr3:uid="{AE341465-00FB-8A48-BD6F-87B7EDC613F6}" name="RMSE"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{3135E420-3270-DF42-A398-9D6F51201E5B}" name="Table6" displayName="Table6" ref="M3:P11" totalsRowShown="0">
-  <autoFilter ref="M3:P11" xr:uid="{3135E420-3270-DF42-A398-9D6F51201E5B}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{76D0AFDB-393E-5247-8B39-99701CA610D3}" name="Features"/>
-    <tableColumn id="2" xr3:uid="{7FBF54F2-6534-6545-853F-CFE153A9F2B1}" name="Accuracy"/>
-    <tableColumn id="3" xr3:uid="{3831066B-52CA-7542-8F44-D6276E3C47FF}" name="Macro_F1"/>
-    <tableColumn id="4" xr3:uid="{5ACCAC01-C4A5-8C4E-8C33-CDA253F7F68F}" name="Weighted_F1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{09BC6A66-48C6-4E42-A3CE-979C30E365B2}" name="Table11" displayName="Table11" ref="F3:J12" totalsRowShown="0">
+  <autoFilter ref="F3:J12" xr:uid="{09BC6A66-48C6-4E42-A3CE-979C30E365B2}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{40A09C1F-1160-9244-81ED-24A028F6186B}" name="Features"/>
+    <tableColumn id="2" xr3:uid="{5D29014F-6B3F-5C4A-92F6-2E7E08C148E7}" name="Accuracy"/>
+    <tableColumn id="3" xr3:uid="{FC0DED5D-FFFF-D843-B72A-C660CCAB2AF5}" name="F1"/>
+    <tableColumn id="4" xr3:uid="{7FDF51BB-571D-6C4B-8D3C-1A9C0AE8E65C}" name="AUC"/>
+    <tableColumn id="5" xr3:uid="{4D4FBD5D-E32E-1F4C-A9E7-419BCA6D6AE4}" name="PR_AUC"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{311780BE-3F99-CE47-BAB5-D4E86E5415DF}" name="Table7" displayName="Table7" ref="M13:Q23" totalsRowShown="0">
-  <autoFilter ref="M13:Q23" xr:uid="{311780BE-3F99-CE47-BAB5-D4E86E5415DF}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{DA773345-809F-1D47-A5D9-6373436312BE}" name="TrainYears"/>
-    <tableColumn id="2" xr3:uid="{88F9015D-2D06-6F4E-9B34-2D51927D5008}" name="TestYears"/>
-    <tableColumn id="3" xr3:uid="{F1707707-89A6-2F4A-85F5-F72594BCFC61}" name="Accuracy"/>
-    <tableColumn id="4" xr3:uid="{1574897B-13EC-DF4E-AE3D-B034B5DD0366}" name="Macro_F1"/>
-    <tableColumn id="5" xr3:uid="{9F00A3A1-A89B-F24F-9CFD-1CDC83584D2C}" name="Weighted_F1" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{B117C16C-4E0D-F545-8277-11E999D66695}" name="Table12" displayName="Table12" ref="F14:K24" totalsRowShown="0">
+  <autoFilter ref="F14:K24" xr:uid="{B117C16C-4E0D-F545-8277-11E999D66695}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{6564D3F5-DA27-E449-AE57-1A91B8FBACD6}" name="TrainYears"/>
+    <tableColumn id="2" xr3:uid="{0FB24013-5EF0-6941-ACBC-5686ECB0E43F}" name="TestYears" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{B8E75AA7-0EBB-894A-82E3-0266343BC9A5}" name="Accuracy"/>
+    <tableColumn id="4" xr3:uid="{A709A651-A4C7-C346-9948-9AD8C9003875}" name="F1"/>
+    <tableColumn id="5" xr3:uid="{5DA4A7CF-1F5E-914E-A627-31A9ADAB8D47}" name="AUC"/>
+    <tableColumn id="6" xr3:uid="{7FBE983D-B457-974B-A0F9-4F17745FE378}" name="PR_AUC" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{8A4D0412-7345-4446-BAEF-22150EB5888A}" name="Table8" displayName="Table8" ref="M26:O34" totalsRowShown="0">
-  <autoFilter ref="M26:O34" xr:uid="{8A4D0412-7345-4446-BAEF-22150EB5888A}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{4734D870-65F8-144E-AF2D-1614B89DA780}" name="Features"/>
-    <tableColumn id="2" xr3:uid="{703B1375-A30E-C243-8B29-2E343DA1DB59}" name="MAE"/>
-    <tableColumn id="3" xr3:uid="{B3C6C8EF-D71A-9A47-812E-58C86A31B52E}" name="RMSE"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8ED91AE2-2535-804F-ADF8-4594327F0593}" name="Table2" displayName="Table2" ref="F27:J36" totalsRowShown="0">
+  <autoFilter ref="F27:J36" xr:uid="{8ED91AE2-2535-804F-ADF8-4594327F0593}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{9CE49F90-F2E3-EB41-B855-2A0215AD85D0}" name="Features"/>
+    <tableColumn id="2" xr3:uid="{4C9AF9A6-5FA5-004C-A20C-E5D33C91C47C}" name="Accuracy"/>
+    <tableColumn id="3" xr3:uid="{743EC3B9-30D6-FA48-A82C-745A3735332D}" name="F1"/>
+    <tableColumn id="4" xr3:uid="{F00EC1B3-C35E-E642-A334-7D745DF09E3B}" name="AUC"/>
+    <tableColumn id="5" xr3:uid="{016C0499-5559-AA4F-8E66-3B6FDA382FE2}" name="PR_AUC"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2434C517-937C-0E4D-91BF-1BD1C677D16F}" name="Table9" displayName="Table9" ref="M36:P46" totalsRowShown="0">
-  <autoFilter ref="M36:P46" xr:uid="{2434C517-937C-0E4D-91BF-1BD1C677D16F}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E81D4BB2-2FFE-5D45-8150-F8BB9C1E47E5}" name="TrainYears"/>
-    <tableColumn id="2" xr3:uid="{3C6762E2-0728-9249-9D96-982E4C1216D6}" name="TestYears"/>
-    <tableColumn id="3" xr3:uid="{3A5CEADE-F36E-CC4E-9BD1-551884B1A47B}" name="MAE"/>
-    <tableColumn id="4" xr3:uid="{D53293EE-83B5-484D-ADA4-6A78FFB8528A}" name="RMSE"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{180CD714-A5AA-CA4F-A4B4-820AA5CCEE8E}" name="Table3" displayName="Table3" ref="F38:K48" totalsRowShown="0">
+  <autoFilter ref="F38:K48" xr:uid="{180CD714-A5AA-CA4F-A4B4-820AA5CCEE8E}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{92824FD7-0B58-B54D-A70E-740BE919A586}" name="TrainYears"/>
+    <tableColumn id="2" xr3:uid="{7C2BD1C1-DE20-974D-91DB-96F5848DB66A}" name="TestYears" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{2CF4DA6C-01C1-2641-BC02-63A926E1A05D}" name="Accuracy"/>
+    <tableColumn id="4" xr3:uid="{E6014188-FD49-CD48-A488-5D7E5663D47F}" name="F1"/>
+    <tableColumn id="5" xr3:uid="{96FA8905-EBE5-3342-B027-439AFA2F0036}" name="AUC"/>
+    <tableColumn id="6" xr3:uid="{4695A5F6-6B01-7641-836E-DC85C1B05D09}" name="PR_AUC"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{A665D967-6C49-E348-BB78-5EEB3FD96D24}" name="Table10" displayName="Table10" ref="M49:O57" totalsRowShown="0">
-  <autoFilter ref="M49:O57" xr:uid="{A665D967-6C49-E348-BB78-5EEB3FD96D24}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B43AE27C-DDD0-EA41-8039-38A3F8DED47D}" name="Features"/>
-    <tableColumn id="2" xr3:uid="{F306D1E8-D371-2542-AC55-840AB710427A}" name="MAE"/>
-    <tableColumn id="3" xr3:uid="{F5C1717C-A6E5-6E43-B11D-BCEC8490F41C}" name="RMSE"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1B783916-8793-1E4C-B01B-F0AE4E13711F}" name="Table4" displayName="Table4" ref="M3:P11" totalsRowShown="0">
+  <autoFilter ref="M3:P11" xr:uid="{1B783916-8793-1E4C-B01B-F0AE4E13711F}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{103C6E61-5DB4-AA4D-90BA-A877D093B450}" name="Features"/>
+    <tableColumn id="2" xr3:uid="{5FBF5494-9C34-FB45-939E-08D5E0ECD6F4}" name="Accuracy"/>
+    <tableColumn id="3" xr3:uid="{5B88A2CF-B89E-9E4E-9F87-B4A862229AFD}" name="Macro_F1"/>
+    <tableColumn id="4" xr3:uid="{0BF817E0-5B5E-A641-B8D6-A67A189E9021}" name="Weighted_F1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -989,7 +949,7 @@
     <col min="11" max="11" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.6640625" customWidth="1"/>
+    <col min="14" max="14" width="19.83203125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.5" customWidth="1"/>
     <col min="16" max="16" width="14.1640625" customWidth="1"/>
     <col min="17" max="17" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -1021,11 +981,11 @@
         <v>2</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K2" s="8"/>
       <c r="M2" s="8" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="Q2" s="8"/>
     </row>
@@ -1036,10 +996,10 @@
       </c>
       <c r="C3" s="2"/>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H3" t="s">
         <v>49</v>
@@ -1048,19 +1008,19 @@
         <v>50</v>
       </c>
       <c r="J3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="M3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O3" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="P3" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
@@ -1070,31 +1030,31 @@
       </c>
       <c r="C4" s="2"/>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G4">
-        <v>0.552014</v>
+        <v>0.46125500000000003</v>
       </c>
       <c r="H4">
-        <v>6.5404000000000004E-2</v>
+        <v>6.5107999999999999E-2</v>
       </c>
       <c r="I4">
-        <v>0.57941100000000001</v>
+        <v>0.58928800000000003</v>
       </c>
       <c r="J4">
-        <v>8.3398E-2</v>
+        <v>3.9300000000000002E-2</v>
       </c>
       <c r="M4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N4">
-        <v>0.75739999999999996</v>
+        <v>0.761571</v>
       </c>
       <c r="O4">
-        <v>0.30444100000000002</v>
+        <v>0.29391</v>
       </c>
       <c r="P4">
-        <v>0.66918900000000003</v>
+        <v>0.66491100000000003</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
@@ -1107,28 +1067,28 @@
         <v>51</v>
       </c>
       <c r="G5">
-        <v>0.96509699999999998</v>
+        <v>0.96845000000000003</v>
       </c>
       <c r="H5">
-        <v>0.33663399999999999</v>
+        <v>0.338065</v>
       </c>
       <c r="I5">
-        <v>0.77165499999999998</v>
+        <v>0.77634899999999996</v>
       </c>
       <c r="J5">
-        <v>0.27485900000000002</v>
+        <v>0.28329900000000002</v>
       </c>
       <c r="M5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N5">
-        <v>0.91172299999999995</v>
+        <v>0.76080099999999995</v>
       </c>
       <c r="O5">
-        <v>0.82779100000000005</v>
+        <v>0.33259100000000003</v>
       </c>
       <c r="P5">
-        <v>0.90869999999999995</v>
+        <v>0.68287900000000001</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
@@ -1138,31 +1098,31 @@
       </c>
       <c r="C6" s="2"/>
       <c r="F6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G6">
-        <v>0.968005</v>
+        <v>0.96519100000000002</v>
       </c>
       <c r="H6">
-        <v>0.33799200000000001</v>
+        <v>0.338785</v>
       </c>
       <c r="I6">
-        <v>0.77957200000000004</v>
+        <v>0.77892700000000004</v>
       </c>
       <c r="J6">
-        <v>0.27460800000000002</v>
+        <v>0.280113</v>
       </c>
       <c r="M6" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="N6">
-        <v>0.91166199999999997</v>
+        <v>0.76080099999999995</v>
       </c>
       <c r="O6">
-        <v>0.82837000000000005</v>
+        <v>0.33259100000000003</v>
       </c>
       <c r="P6">
-        <v>0.90864400000000001</v>
+        <v>0.68287900000000001</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
@@ -1172,31 +1132,31 @@
       </c>
       <c r="C7" s="2"/>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="G7">
-        <v>0.96772899999999995</v>
+        <v>0.96817299999999995</v>
       </c>
       <c r="H7">
-        <v>0.33857799999999999</v>
+        <v>0.34202199999999999</v>
       </c>
       <c r="I7">
-        <v>0.78398500000000004</v>
+        <v>0.78831099999999998</v>
       </c>
       <c r="J7">
-        <v>0.27694200000000002</v>
+        <v>0.28749200000000003</v>
       </c>
       <c r="M7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N7">
-        <v>0.91166199999999997</v>
+        <v>0.76027800000000001</v>
       </c>
       <c r="O7">
-        <v>0.82851200000000003</v>
+        <v>0.33414199999999999</v>
       </c>
       <c r="P7">
-        <v>0.90861999999999998</v>
+        <v>0.681535</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1206,31 +1166,31 @@
       </c>
       <c r="C8" s="3"/>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G8">
-        <v>0.96299999999999997</v>
+        <v>0.967866</v>
       </c>
       <c r="H8">
-        <v>0.33240999999999998</v>
+        <v>0.33818900000000002</v>
       </c>
       <c r="I8">
-        <v>0.78416699999999995</v>
+        <v>0.78885700000000003</v>
       </c>
       <c r="J8">
-        <v>0.27557399999999999</v>
+        <v>0.280221</v>
       </c>
       <c r="M8" t="s">
         <v>43</v>
       </c>
       <c r="N8">
-        <v>0.91184600000000005</v>
+        <v>0.76055499999999998</v>
       </c>
       <c r="O8">
-        <v>0.82949099999999998</v>
+        <v>0.335891</v>
       </c>
       <c r="P8">
-        <v>0.90886299999999998</v>
+        <v>0.68362800000000001</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
@@ -1244,31 +1204,31 @@
         <v>21</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G9">
-        <v>0.96524200000000004</v>
+        <v>0.96820399999999995</v>
       </c>
       <c r="H9">
-        <v>0.34262500000000001</v>
+        <v>0.34307500000000002</v>
       </c>
       <c r="I9">
-        <v>0.784613</v>
+        <v>0.78928799999999999</v>
       </c>
       <c r="J9">
-        <v>0.27930199999999999</v>
+        <v>0.28498899999999999</v>
       </c>
       <c r="M9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N9">
-        <v>0.91310500000000006</v>
+        <v>0.76083199999999995</v>
       </c>
       <c r="O9">
-        <v>0.83079899999999995</v>
+        <v>0.336814</v>
       </c>
       <c r="P9">
-        <v>0.91010400000000002</v>
+        <v>0.68570799999999998</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
@@ -1278,31 +1238,31 @@
       </c>
       <c r="C10" s="2"/>
       <c r="F10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G10">
-        <v>0.96775999999999995</v>
+        <v>0.96688200000000002</v>
       </c>
       <c r="H10">
-        <v>0.336283</v>
+        <v>0.34128399999999998</v>
       </c>
       <c r="I10">
-        <v>0.78576400000000002</v>
+        <v>0.78991199999999995</v>
       </c>
       <c r="J10">
-        <v>0.26985399999999998</v>
+        <v>0.28566399999999997</v>
       </c>
       <c r="M10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N10">
-        <v>0.91411799999999999</v>
+        <v>0.761324</v>
       </c>
       <c r="O10">
-        <v>0.83305099999999999</v>
+        <v>0.33732099999999998</v>
       </c>
       <c r="P10">
-        <v>0.91105199999999997</v>
+        <v>0.68471000000000004</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
@@ -1315,28 +1275,28 @@
         <v>45</v>
       </c>
       <c r="G11">
-        <v>0.966839</v>
+        <v>0.96620499999999998</v>
       </c>
       <c r="H11">
-        <v>0.33660899999999999</v>
+        <v>0.33755299999999999</v>
       </c>
       <c r="I11">
-        <v>0.78839099999999995</v>
+        <v>0.79003599999999996</v>
       </c>
       <c r="J11">
-        <v>0.28140500000000002</v>
+        <v>0.28712700000000002</v>
       </c>
       <c r="M11" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="N11">
-        <v>0.91411799999999999</v>
+        <v>0.76058599999999998</v>
       </c>
       <c r="O11">
-        <v>0.83305099999999999</v>
+        <v>0.33746599999999999</v>
       </c>
       <c r="P11">
-        <v>0.91105199999999997</v>
+        <v>0.684473</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
@@ -1349,16 +1309,16 @@
         <v>44</v>
       </c>
       <c r="G12">
-        <v>0.96607100000000001</v>
+        <v>0.96811199999999997</v>
       </c>
       <c r="H12">
-        <v>0.33713300000000002</v>
+        <v>0.330536</v>
       </c>
       <c r="I12">
-        <v>0.79135200000000006</v>
+        <v>0.79103299999999999</v>
       </c>
       <c r="J12">
-        <v>0.27434399999999998</v>
+        <v>0.28213100000000002</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
@@ -1375,13 +1335,13 @@
         <v>53</v>
       </c>
       <c r="O13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="P13" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="Q13" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
@@ -1397,7 +1357,7 @@
         <v>53</v>
       </c>
       <c r="H14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I14" t="s">
         <v>49</v>
@@ -1406,22 +1366,22 @@
         <v>50</v>
       </c>
       <c r="K14" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="M14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N14" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="O14">
-        <v>0.87639299999999998</v>
+        <v>0.64291900000000002</v>
       </c>
       <c r="P14">
-        <v>0.82737300000000003</v>
+        <v>0.40266400000000002</v>
       </c>
       <c r="Q14">
-        <v>0.87400999999999995</v>
+        <v>0.60002100000000003</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
@@ -1431,38 +1391,38 @@
       </c>
       <c r="C15" s="2"/>
       <c r="F15" t="s">
-        <v>61</v>
-      </c>
-      <c r="G15" s="13">
-        <v>2013</v>
+        <v>59</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="H15">
-        <v>0.96094599999999997</v>
+        <v>0.96038100000000004</v>
       </c>
       <c r="I15">
-        <v>0.43571100000000001</v>
+        <v>0.43063800000000002</v>
       </c>
       <c r="J15">
-        <v>0.84352199999999999</v>
+        <v>0.844198</v>
       </c>
       <c r="K15" s="10">
-        <v>0.42067599999999999</v>
+        <v>0.41855799999999999</v>
       </c>
       <c r="L15" s="10"/>
       <c r="M15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N15" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="O15">
-        <v>0.86777499999999996</v>
+        <v>0.61935399999999996</v>
       </c>
       <c r="P15">
-        <v>0.82509900000000003</v>
+        <v>0.38545499999999999</v>
       </c>
       <c r="Q15">
-        <v>0.86524900000000005</v>
+        <v>0.57023599999999997</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1472,38 +1432,38 @@
       </c>
       <c r="C16" s="3"/>
       <c r="F16" t="s">
-        <v>61</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>66</v>
+        <v>59</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>72</v>
       </c>
       <c r="H16">
-        <v>0.961843</v>
+        <v>0.96141500000000002</v>
       </c>
       <c r="I16">
-        <v>0.39277400000000001</v>
+        <v>0.38882499999999998</v>
       </c>
       <c r="J16">
-        <v>0.80416200000000004</v>
+        <v>0.80419099999999999</v>
       </c>
       <c r="K16" s="10">
-        <v>0.367981</v>
+        <v>0.36621700000000001</v>
       </c>
       <c r="L16" s="10"/>
       <c r="M16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N16" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="O16">
-        <v>0.86243199999999998</v>
+        <v>0.60419400000000001</v>
       </c>
       <c r="P16">
-        <v>0.82362999999999997</v>
+        <v>0.38386100000000001</v>
       </c>
       <c r="Q16" s="10">
-        <v>0.85992999999999997</v>
+        <v>0.55493199999999998</v>
       </c>
       <c r="R16" s="10"/>
     </row>
@@ -1518,38 +1478,38 @@
         <v>25</v>
       </c>
       <c r="F17" t="s">
-        <v>61</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>65</v>
+        <v>59</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>73</v>
       </c>
       <c r="H17">
-        <v>0.95930599999999999</v>
+        <v>0.95894199999999996</v>
       </c>
       <c r="I17">
-        <v>0.36197600000000002</v>
+        <v>0.35651300000000002</v>
       </c>
       <c r="J17">
-        <v>0.783694</v>
+        <v>0.78336899999999998</v>
       </c>
       <c r="K17" s="10">
-        <v>0.34130300000000002</v>
+        <v>0.33648099999999997</v>
       </c>
       <c r="L17" s="10"/>
       <c r="M17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N17" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="O17">
-        <v>0.87315399999999999</v>
+        <v>0.63962600000000003</v>
       </c>
       <c r="P17">
-        <v>0.82397200000000004</v>
+        <v>0.38600600000000002</v>
       </c>
       <c r="Q17" s="10">
-        <v>0.87071699999999996</v>
+        <v>0.59285299999999996</v>
       </c>
       <c r="R17" s="10"/>
     </row>
@@ -1560,38 +1520,38 @@
       </c>
       <c r="C18" s="3"/>
       <c r="F18" t="s">
-        <v>61</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>67</v>
+        <v>59</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="H18">
-        <v>0.96584199999999998</v>
+        <v>0.96544200000000002</v>
       </c>
       <c r="I18">
-        <v>0.351466</v>
+        <v>0.34587600000000002</v>
       </c>
       <c r="J18">
-        <v>0.781474</v>
+        <v>0.78127100000000005</v>
       </c>
       <c r="K18" s="10">
-        <v>0.32487700000000003</v>
+        <v>0.319718</v>
       </c>
       <c r="L18" s="10"/>
       <c r="M18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N18" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="O18">
-        <v>0.85781399999999997</v>
+        <v>0.59073500000000001</v>
       </c>
       <c r="P18">
-        <v>0.82391499999999995</v>
+        <v>0.36030400000000001</v>
       </c>
       <c r="Q18" s="10">
-        <v>0.85473600000000005</v>
+        <v>0.52138499999999999</v>
       </c>
       <c r="R18" s="10"/>
     </row>
@@ -1606,38 +1566,38 @@
         <v>31</v>
       </c>
       <c r="F19" t="s">
-        <v>62</v>
-      </c>
-      <c r="G19" s="13">
-        <v>2014</v>
+        <v>60</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>69</v>
       </c>
       <c r="H19">
-        <v>0.95222300000000004</v>
+        <v>0.95127600000000001</v>
       </c>
       <c r="I19">
-        <v>0.401866</v>
+        <v>0.389349</v>
       </c>
       <c r="J19">
-        <v>0.79334199999999999</v>
+        <v>0.79562600000000006</v>
       </c>
       <c r="K19" s="10">
-        <v>0.38847700000000002</v>
+        <v>0.38270100000000001</v>
       </c>
       <c r="L19" s="10"/>
       <c r="M19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N19" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="O19">
-        <v>0.85403700000000005</v>
+        <v>0.57794699999999999</v>
       </c>
       <c r="P19">
-        <v>0.82218199999999997</v>
+        <v>0.36720399999999997</v>
       </c>
       <c r="Q19" s="10">
-        <v>0.85102699999999998</v>
+        <v>0.51336099999999996</v>
       </c>
       <c r="R19" s="10"/>
     </row>
@@ -1648,38 +1608,38 @@
       </c>
       <c r="C20" s="2"/>
       <c r="F20" t="s">
-        <v>62</v>
-      </c>
-      <c r="G20" s="13" t="s">
-        <v>68</v>
+        <v>60</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>75</v>
       </c>
       <c r="H20">
-        <v>0.94726500000000002</v>
+        <v>0.94662400000000002</v>
       </c>
       <c r="I20">
-        <v>0.38039600000000001</v>
+        <v>0.37202299999999999</v>
       </c>
       <c r="J20">
-        <v>0.78617899999999996</v>
+        <v>0.78626399999999996</v>
       </c>
       <c r="K20" s="10">
-        <v>0.374699</v>
+        <v>0.37044700000000003</v>
       </c>
       <c r="L20" s="10"/>
       <c r="M20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N20" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="O20">
-        <v>0.87051400000000001</v>
+        <v>0.63437900000000003</v>
       </c>
       <c r="P20">
-        <v>0.82530099999999995</v>
+        <v>0.37383100000000002</v>
       </c>
       <c r="Q20" s="10">
-        <v>0.86767099999999997</v>
+        <v>0.57248100000000002</v>
       </c>
       <c r="R20" s="10"/>
     </row>
@@ -1690,38 +1650,38 @@
       </c>
       <c r="C21" s="2"/>
       <c r="F21" t="s">
-        <v>62</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>69</v>
+        <v>60</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="H21">
-        <v>0.95750999999999997</v>
+        <v>0.95708300000000002</v>
       </c>
       <c r="I21">
-        <v>0.36197800000000002</v>
+        <v>0.35461900000000002</v>
       </c>
       <c r="J21">
-        <v>0.77490300000000001</v>
+        <v>0.77535399999999999</v>
       </c>
       <c r="K21" s="10">
-        <v>0.343032</v>
+        <v>0.33985500000000002</v>
       </c>
       <c r="L21" s="10"/>
       <c r="M21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N21" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="O21">
-        <v>0.85951200000000005</v>
+        <v>0.57367599999999996</v>
       </c>
       <c r="P21">
-        <v>0.83225300000000002</v>
+        <v>0.36160300000000001</v>
       </c>
       <c r="Q21" s="10">
-        <v>0.85621999999999998</v>
+        <v>0.49603900000000001</v>
       </c>
       <c r="R21" s="10"/>
     </row>
@@ -1732,38 +1692,38 @@
       </c>
       <c r="C22" s="3"/>
       <c r="F22" t="s">
-        <v>63</v>
-      </c>
-      <c r="G22" s="13">
-        <v>2015</v>
+        <v>61</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="H22">
-        <v>0.93239799999999995</v>
+        <v>0.93305099999999996</v>
       </c>
       <c r="I22">
-        <v>0.376471</v>
+        <v>0.38772099999999998</v>
       </c>
       <c r="J22">
-        <v>0.78699200000000002</v>
+        <v>0.78730100000000003</v>
       </c>
       <c r="K22" s="10">
-        <v>0.38975799999999999</v>
+        <v>0.39171</v>
       </c>
       <c r="L22" s="10"/>
       <c r="M22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N22" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="O22">
-        <v>0.88567700000000005</v>
+        <v>0.67261300000000002</v>
       </c>
       <c r="P22">
-        <v>0.83506999999999998</v>
+        <v>0.36635200000000001</v>
       </c>
       <c r="Q22" s="10">
-        <v>0.88234000000000001</v>
+        <v>0.59509800000000002</v>
       </c>
       <c r="R22" s="10"/>
     </row>
@@ -1778,38 +1738,38 @@
         <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>63</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>70</v>
+        <v>61</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>77</v>
       </c>
       <c r="H23">
-        <v>0.95486800000000005</v>
+        <v>0.95489999999999997</v>
       </c>
       <c r="I23">
-        <v>0.35372599999999998</v>
+        <v>0.35768299999999997</v>
       </c>
       <c r="J23">
-        <v>0.78793999999999997</v>
+        <v>0.78904300000000005</v>
       </c>
       <c r="K23" s="10">
-        <v>0.34151700000000002</v>
+        <v>0.34344799999999998</v>
       </c>
       <c r="L23" s="10"/>
       <c r="M23" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N23" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="O23">
-        <v>0.91114799999999996</v>
+        <v>0.75843499999999997</v>
       </c>
       <c r="P23">
-        <v>0.82787100000000002</v>
+        <v>0.33199499999999998</v>
       </c>
       <c r="Q23" s="10">
-        <v>0.908169</v>
+        <v>0.68051700000000004</v>
       </c>
       <c r="R23" s="10"/>
     </row>
@@ -1820,22 +1780,22 @@
       </c>
       <c r="C24" s="2"/>
       <c r="F24" t="s">
-        <v>64</v>
-      </c>
-      <c r="G24" s="13">
-        <v>2016</v>
+        <v>62</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>71</v>
       </c>
       <c r="H24">
-        <v>0.97039200000000003</v>
+        <v>0.97436299999999998</v>
       </c>
       <c r="I24">
-        <v>0.32036900000000001</v>
+        <v>0.31291600000000003</v>
       </c>
       <c r="J24">
-        <v>0.77261999999999997</v>
+        <v>0.76970400000000005</v>
       </c>
       <c r="K24" s="10">
-        <v>0.27460600000000002</v>
+        <v>0.26910899999999999</v>
       </c>
       <c r="L24" s="10"/>
       <c r="Q24" s="10"/>
@@ -1850,7 +1810,7 @@
       <c r="K25" s="10"/>
       <c r="L25" s="10"/>
       <c r="M25" s="8" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
@@ -1866,12 +1826,12 @@
         <v>40</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
       <c r="M26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N26" t="s">
         <v>41</v>
@@ -1887,56 +1847,56 @@
       </c>
       <c r="C27" s="3"/>
       <c r="F27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H27" t="s">
         <v>49</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="J27" s="10" t="s">
-        <v>72</v>
+      <c r="J27" t="s">
+        <v>64</v>
       </c>
       <c r="L27" s="10"/>
       <c r="M27" t="s">
         <v>44</v>
       </c>
       <c r="N27">
-        <v>21.356171</v>
+        <v>21.331063</v>
       </c>
       <c r="O27">
-        <v>40.147720999999997</v>
+        <v>40.018388000000002</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F28" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G28">
-        <v>0.72571799999999997</v>
+        <v>0.76519999999999999</v>
       </c>
       <c r="H28">
-        <v>1.6733000000000001E-2</v>
-      </c>
-      <c r="I28">
-        <v>0.55503400000000003</v>
-      </c>
-      <c r="J28" s="10">
-        <v>9.1629999999999993E-3</v>
+        <v>1.6480000000000002E-2</v>
+      </c>
+      <c r="I28" s="10">
+        <v>0.55325199999999997</v>
+      </c>
+      <c r="J28">
+        <v>9.2779999999999998E-3</v>
       </c>
       <c r="L28" s="10"/>
       <c r="M28" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="N28">
-        <v>21.356171</v>
+        <v>21.331063</v>
       </c>
       <c r="O28">
-        <v>40.147720999999997</v>
+        <v>40.018388000000002</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
@@ -1944,106 +1904,106 @@
         <v>48</v>
       </c>
       <c r="G29">
-        <v>0.988147</v>
+        <v>0.98745300000000003</v>
       </c>
       <c r="H29">
-        <v>0.45938400000000001</v>
-      </c>
-      <c r="I29">
-        <v>0.99033000000000004</v>
-      </c>
-      <c r="J29" s="10">
-        <v>0.44740799999999997</v>
+        <v>0.44565199999999999</v>
+      </c>
+      <c r="I29" s="10">
+        <v>0.99024299999999998</v>
+      </c>
+      <c r="J29">
+        <v>0.46818100000000001</v>
       </c>
       <c r="L29" s="10"/>
       <c r="M29" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N29">
-        <v>21.562109</v>
+        <v>21.573408000000001</v>
       </c>
       <c r="O29">
-        <v>43.833385999999997</v>
+        <v>40.621310000000001</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F30" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G30">
-        <v>0.99057300000000004</v>
+        <v>0.98806799999999995</v>
       </c>
       <c r="H30">
-        <v>0.492562</v>
-      </c>
-      <c r="I30">
-        <v>0.99037299999999995</v>
-      </c>
-      <c r="J30" s="10">
-        <v>0.45460800000000001</v>
+        <v>0.45197700000000002</v>
+      </c>
+      <c r="I30" s="10">
+        <v>0.99029900000000004</v>
+      </c>
+      <c r="J30">
+        <v>0.47044799999999998</v>
       </c>
       <c r="L30" s="10"/>
       <c r="M30" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="N30">
-        <v>21.727955000000001</v>
+        <v>21.699954999999999</v>
       </c>
       <c r="O30">
-        <v>45.345025999999997</v>
+        <v>44.431638999999997</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F31" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G31">
-        <v>0.98713300000000004</v>
+        <v>0.98425399999999996</v>
       </c>
       <c r="H31">
-        <v>0.45513700000000001</v>
-      </c>
-      <c r="I31">
-        <v>0.990649</v>
-      </c>
-      <c r="J31" s="10">
-        <v>0.445687</v>
+        <v>0.414188</v>
+      </c>
+      <c r="I31" s="10">
+        <v>0.99034299999999997</v>
+      </c>
+      <c r="J31">
+        <v>0.45035199999999997</v>
       </c>
       <c r="L31" s="10"/>
       <c r="M31" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N31">
-        <v>21.748033</v>
+        <v>21.761336</v>
       </c>
       <c r="O31">
-        <v>44.856802000000002</v>
+        <v>44.335087000000001</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F32" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="G32">
-        <v>0.98774799999999996</v>
+        <v>0.991174</v>
       </c>
       <c r="H32">
-        <v>0.461538</v>
+        <v>0.50431800000000004</v>
       </c>
       <c r="I32">
-        <v>0.990699</v>
+        <v>0.99044100000000002</v>
       </c>
       <c r="J32">
-        <v>0.45185799999999998</v>
+        <v>0.490645</v>
       </c>
       <c r="M32" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="N32">
-        <v>21.753784</v>
+        <v>21.798490999999999</v>
       </c>
       <c r="O32">
-        <v>45.101326</v>
+        <v>45.202117000000001</v>
       </c>
     </row>
     <row r="33" spans="6:16" x14ac:dyDescent="0.2">
@@ -2051,68 +2011,68 @@
         <v>46</v>
       </c>
       <c r="G33">
-        <v>0.98780900000000005</v>
+        <v>0.98696099999999998</v>
       </c>
       <c r="H33">
-        <v>0.45839000000000002</v>
+        <v>0.44357000000000002</v>
       </c>
       <c r="I33">
-        <v>0.99074099999999998</v>
+        <v>0.99048400000000003</v>
       </c>
       <c r="J33">
-        <v>0.45094600000000001</v>
+        <v>0.47344700000000001</v>
       </c>
       <c r="M33" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="N33">
-        <v>21.810227999999999</v>
+        <v>21.844002</v>
       </c>
       <c r="O33">
-        <v>41.057747999999997</v>
+        <v>45.109938</v>
       </c>
     </row>
     <row r="34" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F34" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="G34">
-        <v>0.98774799999999996</v>
+        <v>0.99169700000000005</v>
       </c>
       <c r="H34">
-        <v>0.46298800000000001</v>
+        <v>0.50367600000000001</v>
       </c>
       <c r="I34">
-        <v>0.99112699999999998</v>
+        <v>0.99053199999999997</v>
       </c>
       <c r="J34">
-        <v>0.488319</v>
+        <v>0.47437699999999999</v>
       </c>
       <c r="M34" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N34">
-        <v>29.966094999999999</v>
+        <v>22.042000000000002</v>
       </c>
       <c r="O34">
-        <v>50.354850999999996</v>
+        <v>44.435901999999999</v>
       </c>
     </row>
     <row r="35" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F35" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G35">
-        <v>0.991371</v>
+        <v>0.991174</v>
       </c>
       <c r="H35">
-        <v>0.51130399999999998</v>
+        <v>0.47912900000000003</v>
       </c>
       <c r="I35">
-        <v>0.99120299999999995</v>
+        <v>0.99054200000000003</v>
       </c>
       <c r="J35">
-        <v>0.45757500000000001</v>
+        <v>0.46995100000000001</v>
       </c>
     </row>
     <row r="36" spans="6:16" x14ac:dyDescent="0.2">
@@ -2120,16 +2080,16 @@
         <v>44</v>
       </c>
       <c r="G36">
-        <v>0.98774799999999996</v>
+        <v>0.98711400000000005</v>
       </c>
       <c r="H36">
-        <v>0.46443000000000001</v>
+        <v>0.44795800000000002</v>
       </c>
       <c r="I36">
-        <v>0.99126199999999998</v>
+        <v>0.99080999999999997</v>
       </c>
       <c r="J36">
-        <v>0.50215200000000004</v>
+        <v>0.50368100000000005</v>
       </c>
       <c r="M36" t="s">
         <v>52</v>
@@ -2146,16 +2106,16 @@
     </row>
     <row r="37" spans="6:16" x14ac:dyDescent="0.2">
       <c r="M37" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N37" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="O37">
-        <v>28.937231000000001</v>
+        <v>28.915358999999999</v>
       </c>
       <c r="P37">
-        <v>57.185696</v>
+        <v>57.130614999999999</v>
       </c>
     </row>
     <row r="38" spans="6:16" x14ac:dyDescent="0.2">
@@ -2166,7 +2126,7 @@
         <v>53</v>
       </c>
       <c r="H38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I38" t="s">
         <v>49</v>
@@ -2175,323 +2135,323 @@
         <v>50</v>
       </c>
       <c r="K38" t="s">
+        <v>64</v>
+      </c>
+      <c r="M38" t="s">
+        <v>59</v>
+      </c>
+      <c r="N38" t="s">
         <v>72</v>
       </c>
-      <c r="M38" t="s">
-        <v>61</v>
-      </c>
-      <c r="N38" t="s">
-        <v>84</v>
-      </c>
       <c r="O38">
-        <v>34.397162000000002</v>
+        <v>34.332116999999997</v>
       </c>
       <c r="P38">
-        <v>101.85309599999999</v>
+        <v>101.74705</v>
       </c>
     </row>
     <row r="39" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F39" t="s">
-        <v>61</v>
-      </c>
-      <c r="G39" s="12">
-        <v>2013</v>
+        <v>59</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="H39">
-        <v>0.96592999999999996</v>
+        <v>0.966499</v>
       </c>
       <c r="I39">
-        <v>0.33793099999999998</v>
+        <v>0.34282400000000002</v>
       </c>
       <c r="J39">
-        <v>0.98298099999999999</v>
+        <v>0.98116599999999998</v>
       </c>
       <c r="K39">
-        <v>0.42547200000000002</v>
+        <v>0.391148</v>
       </c>
       <c r="M39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N39" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="O39">
-        <v>38.008125999999997</v>
+        <v>37.947282999999999</v>
       </c>
       <c r="P39">
-        <v>125.167216</v>
+        <v>125.1007</v>
       </c>
     </row>
     <row r="40" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F40" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H40">
-        <v>0.96802200000000005</v>
+        <v>0.96820200000000001</v>
       </c>
       <c r="I40">
-        <v>0.33884999999999998</v>
+        <v>0.33929100000000001</v>
       </c>
       <c r="J40">
-        <v>0.97485699999999997</v>
+        <v>0.97120300000000004</v>
       </c>
       <c r="K40">
-        <v>0.41587600000000002</v>
+        <v>0.392984</v>
       </c>
       <c r="M40" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N40" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="O40">
-        <v>35.060549000000002</v>
+        <v>34.941094999999997</v>
       </c>
       <c r="P40">
-        <v>109.622733</v>
+        <v>109.5206</v>
       </c>
     </row>
     <row r="41" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F41" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G41" s="12" t="s">
         <v>73</v>
       </c>
       <c r="H41">
-        <v>0.96983699999999995</v>
+        <v>0.96958299999999997</v>
       </c>
       <c r="I41">
-        <v>0.349192</v>
+        <v>0.347632</v>
       </c>
       <c r="J41">
-        <v>0.97384999999999999</v>
+        <v>0.97131599999999996</v>
       </c>
       <c r="K41">
-        <v>0.393675</v>
+        <v>0.37111100000000002</v>
       </c>
       <c r="M41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N41" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="O41">
-        <v>38.333430999999997</v>
+        <v>38.262385999999999</v>
       </c>
       <c r="P41">
-        <v>130.53248099999999</v>
+        <v>130.76484500000001</v>
       </c>
     </row>
     <row r="42" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F42" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G42" s="12" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="H42">
-        <v>0.979939</v>
+        <v>0.97005699999999995</v>
       </c>
       <c r="I42">
-        <v>0.34106599999999998</v>
+        <v>0.33469199999999999</v>
       </c>
       <c r="J42">
-        <v>0.97753800000000002</v>
+        <v>0.97485100000000002</v>
       </c>
       <c r="K42">
-        <v>0.38775599999999999</v>
+        <v>0.36384499999999997</v>
       </c>
       <c r="M42" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N42" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="O42">
-        <v>41.588926999999998</v>
+        <v>41.518132000000001</v>
       </c>
       <c r="P42">
-        <v>148.71897200000001</v>
+        <v>148.90353200000001</v>
       </c>
     </row>
     <row r="43" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F43" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="H43">
-        <v>0.971109</v>
+        <v>0.97206300000000001</v>
       </c>
       <c r="I43">
-        <v>0.34375</v>
+        <v>0.352628</v>
       </c>
       <c r="J43">
-        <v>0.96608099999999997</v>
+        <v>0.96902100000000002</v>
       </c>
       <c r="K43">
-        <v>0.41814699999999999</v>
+        <v>0.43715399999999999</v>
       </c>
       <c r="M43" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N43" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="O43">
-        <v>35.577967000000001</v>
+        <v>35.577832000000001</v>
       </c>
       <c r="P43">
-        <v>121.821141</v>
+        <v>121.936886</v>
       </c>
     </row>
     <row r="44" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G44" s="12" t="s">
         <v>75</v>
       </c>
       <c r="H44">
-        <v>0.97258100000000003</v>
+        <v>0.97291000000000005</v>
       </c>
       <c r="I44">
-        <v>0.35824299999999998</v>
+        <v>0.36232999999999999</v>
       </c>
       <c r="J44">
-        <v>0.97062700000000002</v>
+        <v>0.97276300000000004</v>
       </c>
       <c r="K44">
-        <v>0.40179300000000001</v>
+        <v>0.39738600000000002</v>
       </c>
       <c r="M44" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N44" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="O44">
-        <v>46.294682000000002</v>
+        <v>46.509390000000003</v>
       </c>
       <c r="P44">
-        <v>173.36434600000001</v>
+        <v>173.446901</v>
       </c>
     </row>
     <row r="45" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F45" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G45" s="12" t="s">
         <v>76</v>
       </c>
       <c r="H45">
-        <v>0.97283699999999995</v>
+        <v>0.97327399999999997</v>
       </c>
       <c r="I45">
-        <v>0.34074399999999999</v>
+        <v>0.34635700000000003</v>
       </c>
       <c r="J45">
-        <v>0.97666299999999995</v>
+        <v>0.97862499999999997</v>
       </c>
       <c r="K45">
-        <v>0.396652</v>
+        <v>0.40161200000000002</v>
       </c>
       <c r="M45" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N45" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="O45">
-        <v>33.006653</v>
+        <v>33.024493999999997</v>
       </c>
       <c r="P45">
-        <v>119.331626</v>
+        <v>119.44378</v>
       </c>
     </row>
     <row r="46" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F46" t="s">
-        <v>63</v>
-      </c>
-      <c r="G46" s="12">
-        <v>2015</v>
+        <v>61</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>70</v>
       </c>
       <c r="H46">
-        <v>0.97343199999999996</v>
+        <v>0.97281799999999996</v>
       </c>
       <c r="I46">
-        <v>0.374249</v>
+        <v>0.36917899999999998</v>
       </c>
       <c r="J46">
-        <v>0.97331299999999998</v>
+        <v>0.97289099999999995</v>
       </c>
       <c r="K46">
-        <v>0.36546400000000001</v>
+        <v>0.36420400000000003</v>
       </c>
       <c r="M46" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N46" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="O46">
-        <v>22.270596000000001</v>
+        <v>22.153655000000001</v>
       </c>
       <c r="P46">
-        <v>46.302942000000002</v>
+        <v>45.861156000000001</v>
       </c>
     </row>
     <row r="47" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F47" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="H47">
-        <v>0.97382000000000002</v>
+        <v>0.97269799999999995</v>
       </c>
       <c r="I47">
-        <v>0.34747800000000001</v>
+        <v>0.33827000000000002</v>
       </c>
       <c r="J47">
-        <v>0.98085</v>
+        <v>0.98832200000000003</v>
       </c>
       <c r="K47">
-        <v>0.38545499999999999</v>
+        <v>0.39226899999999998</v>
       </c>
     </row>
     <row r="48" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F48" t="s">
-        <v>64</v>
-      </c>
-      <c r="G48" s="12">
-        <v>2016</v>
+        <v>62</v>
+      </c>
+      <c r="G48" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="H48">
-        <v>0.96843900000000005</v>
+        <v>0.97159700000000004</v>
       </c>
       <c r="I48">
-        <v>0.29050999999999999</v>
+        <v>0.31101800000000002</v>
       </c>
       <c r="J48">
-        <v>0.99012199999999995</v>
+        <v>0.99056900000000003</v>
       </c>
       <c r="K48">
-        <v>0.44844400000000001</v>
+        <v>0.42571900000000001</v>
       </c>
       <c r="M48" s="8" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M49" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N49" t="s">
         <v>41</v>
@@ -2505,87 +2465,87 @@
         <v>44</v>
       </c>
       <c r="N50">
-        <v>4.999771</v>
+        <v>5.046481</v>
       </c>
       <c r="O50">
-        <v>54.533540000000002</v>
+        <v>52.632469</v>
       </c>
     </row>
     <row r="51" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M51" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="N51">
-        <v>4.999771</v>
+        <v>5.046481</v>
       </c>
       <c r="O51">
-        <v>54.533540000000002</v>
+        <v>52.632469</v>
       </c>
     </row>
     <row r="52" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M52" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="N52">
-        <v>5.3214519999999998</v>
+        <v>5.2630610000000004</v>
       </c>
       <c r="O52">
-        <v>49.957478999999999</v>
+        <v>49.904974000000003</v>
       </c>
     </row>
     <row r="53" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M53" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N53">
-        <v>5.3366499999999997</v>
+        <v>5.2900390000000002</v>
       </c>
       <c r="O53">
-        <v>51.564582999999999</v>
+        <v>50.791508999999998</v>
       </c>
     </row>
     <row r="54" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M54" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N54">
-        <v>5.3580769999999998</v>
+        <v>5.3591059999999997</v>
       </c>
       <c r="O54">
-        <v>51.091512000000002</v>
+        <v>50.596747000000001</v>
       </c>
     </row>
     <row r="55" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M55" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="N55">
-        <v>5.4430750000000003</v>
+        <v>5.3799539999999997</v>
       </c>
       <c r="O55">
-        <v>52.723154999999998</v>
+        <v>49.703651000000001</v>
       </c>
     </row>
     <row r="56" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M56" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N56">
-        <v>5.4592210000000003</v>
+        <v>5.48386</v>
       </c>
       <c r="O56">
-        <v>51.699086999999999</v>
+        <v>51.300445000000003</v>
       </c>
     </row>
     <row r="57" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M57" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N57">
-        <v>6.1928089999999996</v>
+        <v>6.2684230000000003</v>
       </c>
       <c r="O57">
-        <v>49.025499000000003</v>
+        <v>47.642814000000001</v>
       </c>
     </row>
     <row r="59" spans="13:16" x14ac:dyDescent="0.2">
@@ -2604,142 +2564,142 @@
     </row>
     <row r="60" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M60" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N60" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="O60">
-        <v>9.8113840000000003</v>
+        <v>9.8770170000000004</v>
       </c>
       <c r="P60">
-        <v>101.43481300000001</v>
+        <v>101.84092099999999</v>
       </c>
     </row>
     <row r="61" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M61" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N61" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="O61">
-        <v>9.5015479999999997</v>
+        <v>9.6460150000000002</v>
       </c>
       <c r="P61">
-        <v>95.078704000000002</v>
+        <v>95.695426999999995</v>
       </c>
     </row>
     <row r="62" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M62" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N62" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="O62">
-        <v>9.1452589999999994</v>
+        <v>9.4155809999999995</v>
       </c>
       <c r="P62">
-        <v>92.305087999999998</v>
+        <v>93.770842999999999</v>
       </c>
     </row>
     <row r="63" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M63" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N63" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="O63">
-        <v>8.5295509999999997</v>
+        <v>8.7875540000000001</v>
       </c>
       <c r="P63">
-        <v>88.275791999999996</v>
+        <v>89.000607000000002</v>
       </c>
     </row>
     <row r="64" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M64" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N64" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="O64">
-        <v>8.8767320000000005</v>
+        <v>9.1319040000000005</v>
       </c>
       <c r="P64">
-        <v>78.271040999999997</v>
+        <v>78.227881999999994</v>
       </c>
     </row>
     <row r="65" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M65" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N65" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="O65">
-        <v>8.5915210000000002</v>
+        <v>8.7785270000000004</v>
       </c>
       <c r="P65">
-        <v>79.835553000000004</v>
+        <v>80.302413000000001</v>
       </c>
     </row>
     <row r="66" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M66" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="N66" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="O66">
-        <v>7.9163309999999996</v>
+        <v>8.04819</v>
       </c>
       <c r="P66">
-        <v>73.733508999999998</v>
+        <v>73.691861000000003</v>
       </c>
     </row>
     <row r="67" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M67" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N67" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="O67">
-        <v>7.3983889999999999</v>
+        <v>7.497763</v>
       </c>
       <c r="P67">
-        <v>78.856120000000004</v>
+        <v>79.516654000000003</v>
       </c>
     </row>
     <row r="68" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M68" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N68" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="O68">
-        <v>6.4303210000000002</v>
+        <v>6.4677600000000002</v>
       </c>
       <c r="P68">
-        <v>65.430160000000001</v>
+        <v>65.158376000000004</v>
       </c>
     </row>
     <row r="69" spans="13:16" x14ac:dyDescent="0.2">
       <c r="M69" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N69" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="O69">
-        <v>5.5630249999999997</v>
+        <v>5.5395760000000003</v>
       </c>
       <c r="P69">
-        <v>46.306967</v>
+        <v>50.761203000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>